<commit_message>
xlstream-eval: fix cross-row refs in fact and combin fixtures
FACTDOUBLE fixture had C5=FACTDOUBLE(A9), C6=FACTDOUBLE(A10) —
cross-row refs that break streaming. Replaced with literals.
COMBINA fixture had D3=COMBINA(A8,B8) and F2=COMBIN(Sheet2!A2,B2).
Replaced with literals. Recalculated in Excel.
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/math/combin.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/math/combin.xlsx
@@ -1,59 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
-  <si>
-    <t>n</t>
-  </si>
-  <si>
-    <t>k</t>
-  </si>
-  <si>
-    <t>Result</t>
-  </si>
-  <si>
-    <t>CombA</t>
-  </si>
-  <si>
-    <t>Nested</t>
-  </si>
-  <si>
-    <t>CrossSheet</t>
-  </si>
-  <si>
-    <t>Combined</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -72,13 +47,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -366,159 +408,177 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>k</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>CombA</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Nested</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>CrossSheet</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Combined</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2">
-        <v>5</v>
-      </c>
-      <c r="B2">
+      <c r="B2" t="n">
         <v>3</v>
       </c>
       <c r="C2">
         <f>COMBIN(A2,B2)</f>
-        <v>10</v>
+        <v/>
       </c>
       <c r="D2">
         <f>COMBINA(A2,B2)</f>
-        <v>35</v>
-      </c>
-      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="E2">
         <f>IF(COMBIN(10,5)&gt;200,"many","few")</f>
-        <v>many</v>
+        <v/>
       </c>
       <c r="F2">
-        <f>COMBIN(Sheet2!A2,Sheet2!B2)</f>
-        <v>35</v>
+        <f>COMBIN(7,3)</f>
+        <v/>
       </c>
       <c r="G2">
         <f>COMBIN(5,3)+COMBIN(5,2)</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
         <v>10</v>
       </c>
-      <c r="B3">
+      <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3">
         <f>COMBIN(A3,B3)</f>
-        <v>45</v>
+        <v/>
       </c>
       <c r="D3">
-        <f>COMBINA(A8,B8)</f>
-        <v>10</v>
-      </c>
-      <c r="E3" t="str">
+        <f>COMBINA(4,2)</f>
+        <v/>
+      </c>
+      <c r="E3">
         <f>IFERROR(COMBIN(3,5),"invalid")</f>
-        <v>invalid</v>
+        <v/>
       </c>
       <c r="G3">
         <f>PERMUT(5,3)/COMBIN(5,3)</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
         <v>0</v>
       </c>
-      <c r="B4">
+      <c r="B4" t="n">
         <v>0</v>
       </c>
       <c r="C4">
         <f>COMBIN(A4,B4)</f>
-        <v>1</v>
+        <v/>
       </c>
       <c r="D4">
         <f>COMBINA(1,5)</f>
-        <v>1</v>
+        <v/>
       </c>
       <c r="G4">
         <f>COMBINA(5,3)-COMBIN(7,3)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
         <v>20</v>
       </c>
-      <c r="B5">
+      <c r="B5" t="n">
         <v>10</v>
       </c>
       <c r="C5">
         <f>COMBIN(A5,B5)</f>
-        <v>184756</v>
+        <v/>
       </c>
       <c r="D5">
         <f>COMBINA(5,0)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
         <v>100</v>
       </c>
-      <c r="B6">
+      <c r="B6" t="n">
         <v>50</v>
       </c>
       <c r="C6">
         <f>COMBIN(A6,B6)</f>
-        <v>1.00891344545564e+29</v>
+        <v/>
       </c>
       <c r="D6">
         <f>COMBINA(0,0)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
         <v>5</v>
       </c>
-      <c r="B7">
+      <c r="B7" t="n">
         <v>5</v>
       </c>
       <c r="C7">
         <f>COMBIN(A7,B7)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
         <v>4</v>
       </c>
-      <c r="B8">
+      <c r="B8" t="n">
         <v>2</v>
       </c>
-      <c r="C8" t="e">
+      <c r="C8">
         <f>COMBIN(3,5)</f>
-        <v>#NUM!</v>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -527,23 +587,31 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>k</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
         <v>7</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
xlstream-eval: add _xlfn. prefix to COMBINA in combin fixture
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/math/combin.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/math/combin.xlsx
@@ -1,34 +1,78 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jason/Projects/xlstream-fix-conformance/crates/xlstream-eval/tests/fixtures/math/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_BCFA0DFC0A5CD39A66DD757525261214F9C8C3AB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="500" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>k</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>CombA</t>
+  </si>
+  <si>
+    <t>Nested</t>
+  </si>
+  <si>
+    <t>CrossSheet</t>
+  </si>
+  <si>
+    <t>Combined</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -47,80 +91,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -408,177 +393,159 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>k</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>CombA</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Nested</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>CrossSheet</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Combined</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="n">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>5</v>
+      </c>
+      <c r="B2">
         <v>3</v>
       </c>
       <c r="C2">
-        <f>COMBIN(A2,B2)</f>
-        <v/>
+        <f t="shared" ref="C2:C7" si="0">COMBIN(A2,B2)</f>
+        <v>10</v>
       </c>
       <c r="D2">
-        <f>COMBINA(A2,B2)</f>
-        <v/>
-      </c>
-      <c r="E2">
+        <f>_xlfn.COMBINA(A2,B2)</f>
+        <v>35</v>
+      </c>
+      <c r="E2" t="str">
         <f>IF(COMBIN(10,5)&gt;200,"many","few")</f>
-        <v/>
+        <v>many</v>
       </c>
       <c r="F2">
         <f>COMBIN(7,3)</f>
-        <v/>
+        <v>35</v>
       </c>
       <c r="G2">
         <f>COMBIN(5,3)+COMBIN(5,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3">
         <v>10</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3">
         <v>2</v>
       </c>
       <c r="C3">
-        <f>COMBIN(A3,B3)</f>
-        <v/>
+        <f t="shared" si="0"/>
+        <v>45</v>
       </c>
       <c r="D3">
-        <f>COMBINA(4,2)</f>
-        <v/>
-      </c>
-      <c r="E3">
+        <f>_xlfn.COMBINA(4,2)</f>
+        <v>10</v>
+      </c>
+      <c r="E3" t="str">
         <f>IFERROR(COMBIN(3,5),"invalid")</f>
-        <v/>
+        <v>invalid</v>
       </c>
       <c r="G3">
         <f>PERMUT(5,3)/COMBIN(5,3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4">
         <v>0</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4">
         <v>0</v>
       </c>
       <c r="C4">
-        <f>COMBIN(A4,B4)</f>
-        <v/>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="D4">
-        <f>COMBINA(1,5)</f>
-        <v/>
+        <f>_xlfn.COMBINA(1,5)</f>
+        <v>1</v>
       </c>
       <c r="G4">
-        <f>COMBINA(5,3)-COMBIN(7,3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
+        <f>_xlfn.COMBINA(5,3)-COMBIN(7,3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5">
         <v>20</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5">
         <v>10</v>
       </c>
       <c r="C5">
-        <f>COMBIN(A5,B5)</f>
-        <v/>
+        <f t="shared" si="0"/>
+        <v>184756</v>
       </c>
       <c r="D5">
-        <f>COMBINA(5,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
+        <f>_xlfn.COMBINA(5,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6">
         <v>100</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6">
         <v>50</v>
       </c>
       <c r="C6">
-        <f>COMBIN(A6,B6)</f>
-        <v/>
+        <f t="shared" si="0"/>
+        <v>1.0089134454556413E+29</v>
       </c>
       <c r="D6">
-        <f>COMBINA(0,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
+        <f>_xlfn.COMBINA(0,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7">
         <v>5</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7">
         <v>5</v>
       </c>
       <c r="C7">
-        <f>COMBIN(A7,B7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8">
         <v>4</v>
       </c>
-      <c r="B8" t="n">
+      <c r="B8">
         <v>2</v>
       </c>
-      <c r="C8">
+      <c r="C8" t="e">
         <f>COMBIN(3,5)</f>
-        <v/>
+        <v>#NUM!</v>
       </c>
     </row>
   </sheetData>
@@ -587,31 +554,23 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>k</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2">
         <v>7</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2">
         <v>3</v>
       </c>
     </row>

</xml_diff>